<commit_message>
Comeback and update the Legend database :v
</commit_message>
<xml_diff>
--- a/excel/player_team_achievements.xlsx
+++ b/excel/player_team_achievements.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="96">
   <si>
     <t>id</t>
   </si>
@@ -64,19 +64,28 @@
     <t>naruto</t>
   </si>
   <si>
+    <t>boruto7SCW2022</t>
+  </si>
+  <si>
+    <t>SC</t>
+  </si>
+  <si>
+    <t>Winter 2022</t>
+  </si>
+  <si>
     <t>dbz1SCW2022</t>
   </si>
   <si>
     <t>dbz_1</t>
   </si>
   <si>
-    <t>SC</t>
-  </si>
-  <si>
     <t>db</t>
   </si>
   <si>
-    <t>Winter 2022</t>
+    <t>dbz1SCS2022</t>
+  </si>
+  <si>
+    <t>Spring 2022</t>
   </si>
   <si>
     <t>dbz1AFC2024</t>
@@ -1473,7 +1482,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="7" width="16.3516" style="1" customWidth="1"/>
@@ -1569,70 +1578,70 @@
         <v>17</v>
       </c>
       <c r="B5" t="s" s="7">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C5" t="s" s="7">
         <v>12</v>
       </c>
       <c r="D5" t="s" s="7">
+        <v>18</v>
+      </c>
+      <c r="E5" t="s" s="7">
+        <v>16</v>
+      </c>
+      <c r="F5" t="s" s="7">
         <v>19</v>
-      </c>
-      <c r="E5" t="s" s="7">
-        <v>20</v>
-      </c>
-      <c r="F5" t="s" s="7">
-        <v>21</v>
       </c>
       <c r="G5" s="9"/>
     </row>
     <row r="6" ht="23.2" customHeight="1">
       <c r="A6" t="s" s="7">
+        <v>20</v>
+      </c>
+      <c r="B6" t="s" s="7">
+        <v>21</v>
+      </c>
+      <c r="C6" t="s" s="7">
+        <v>8</v>
+      </c>
+      <c r="D6" t="s" s="7">
+        <v>18</v>
+      </c>
+      <c r="E6" t="s" s="7">
         <v>22</v>
       </c>
-      <c r="B6" t="s" s="7">
-        <v>18</v>
-      </c>
-      <c r="C6" t="s" s="7">
-        <v>12</v>
-      </c>
-      <c r="D6" t="s" s="7">
-        <v>9</v>
-      </c>
-      <c r="E6" t="s" s="7">
-        <v>23</v>
-      </c>
-      <c r="F6" s="8">
-        <v>2024</v>
+      <c r="F6" t="s" s="7">
+        <v>19</v>
       </c>
       <c r="G6" s="9"/>
     </row>
     <row r="7" ht="23.2" customHeight="1">
       <c r="A7" t="s" s="7">
+        <v>23</v>
+      </c>
+      <c r="B7" t="s" s="7">
+        <v>21</v>
+      </c>
+      <c r="C7" t="s" s="7">
+        <v>8</v>
+      </c>
+      <c r="D7" t="s" s="7">
+        <v>18</v>
+      </c>
+      <c r="E7" t="s" s="7">
+        <v>22</v>
+      </c>
+      <c r="F7" t="s" s="7">
         <v>24</v>
-      </c>
-      <c r="B7" t="s" s="7">
-        <v>25</v>
-      </c>
-      <c r="C7" t="s" s="7">
-        <v>12</v>
-      </c>
-      <c r="D7" t="s" s="7">
-        <v>9</v>
-      </c>
-      <c r="E7" t="s" s="7">
-        <v>23</v>
-      </c>
-      <c r="F7" s="8">
-        <v>2024</v>
       </c>
       <c r="G7" s="9"/>
     </row>
     <row r="8" ht="23.2" customHeight="1">
       <c r="A8" t="s" s="7">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B8" t="s" s="7">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="C8" t="s" s="7">
         <v>12</v>
@@ -1641,7 +1650,7 @@
         <v>9</v>
       </c>
       <c r="E8" t="s" s="7">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F8" s="8">
         <v>2024</v>
@@ -1650,10 +1659,10 @@
     </row>
     <row r="9" ht="23.2" customHeight="1">
       <c r="A9" t="s" s="7">
+        <v>27</v>
+      </c>
+      <c r="B9" t="s" s="7">
         <v>28</v>
-      </c>
-      <c r="B9" t="s" s="7">
-        <v>29</v>
       </c>
       <c r="C9" t="s" s="7">
         <v>12</v>
@@ -1662,7 +1671,7 @@
         <v>9</v>
       </c>
       <c r="E9" t="s" s="7">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F9" s="8">
         <v>2024</v>
@@ -1671,10 +1680,10 @@
     </row>
     <row r="10" ht="23.2" customHeight="1">
       <c r="A10" t="s" s="7">
+        <v>29</v>
+      </c>
+      <c r="B10" t="s" s="7">
         <v>30</v>
-      </c>
-      <c r="B10" t="s" s="7">
-        <v>31</v>
       </c>
       <c r="C10" t="s" s="7">
         <v>12</v>
@@ -1683,7 +1692,7 @@
         <v>9</v>
       </c>
       <c r="E10" t="s" s="7">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F10" s="8">
         <v>2024</v>
@@ -1692,10 +1701,10 @@
     </row>
     <row r="11" ht="23.2" customHeight="1">
       <c r="A11" t="s" s="7">
+        <v>31</v>
+      </c>
+      <c r="B11" t="s" s="7">
         <v>32</v>
-      </c>
-      <c r="B11" t="s" s="7">
-        <v>33</v>
       </c>
       <c r="C11" t="s" s="7">
         <v>12</v>
@@ -1704,7 +1713,7 @@
         <v>9</v>
       </c>
       <c r="E11" t="s" s="7">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F11" s="8">
         <v>2024</v>
@@ -1713,43 +1722,43 @@
     </row>
     <row r="12" ht="23.2" customHeight="1">
       <c r="A12" t="s" s="7">
+        <v>33</v>
+      </c>
+      <c r="B12" t="s" s="7">
         <v>34</v>
       </c>
-      <c r="B12" t="s" s="7">
-        <v>35</v>
-      </c>
       <c r="C12" t="s" s="7">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D12" t="s" s="7">
         <v>9</v>
       </c>
       <c r="E12" t="s" s="7">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F12" s="8">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="G12" s="9"/>
     </row>
     <row r="13" ht="23.2" customHeight="1">
       <c r="A13" t="s" s="7">
+        <v>35</v>
+      </c>
+      <c r="B13" t="s" s="7">
         <v>36</v>
-      </c>
-      <c r="B13" t="s" s="7">
-        <v>35</v>
       </c>
       <c r="C13" t="s" s="7">
         <v>12</v>
       </c>
       <c r="D13" t="s" s="7">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E13" t="s" s="7">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F13" s="8">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="G13" s="9"/>
     </row>
@@ -1758,7 +1767,7 @@
         <v>37</v>
       </c>
       <c r="B14" t="s" s="7">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C14" t="s" s="7">
         <v>8</v>
@@ -1770,28 +1779,28 @@
         <v>10</v>
       </c>
       <c r="F14" s="8">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="G14" s="9"/>
     </row>
     <row r="15" ht="23.2" customHeight="1">
       <c r="A15" t="s" s="7">
+        <v>39</v>
+      </c>
+      <c r="B15" t="s" s="7">
         <v>38</v>
       </c>
-      <c r="B15" t="s" s="7">
-        <v>39</v>
-      </c>
       <c r="C15" t="s" s="7">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D15" t="s" s="7">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E15" t="s" s="7">
         <v>10</v>
       </c>
       <c r="F15" s="8">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="G15" s="9"/>
     </row>
@@ -1800,7 +1809,7 @@
         <v>40</v>
       </c>
       <c r="B16" t="s" s="7">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C16" t="s" s="7">
         <v>8</v>
@@ -1818,10 +1827,10 @@
     </row>
     <row r="17" ht="23.2" customHeight="1">
       <c r="A17" t="s" s="7">
+        <v>41</v>
+      </c>
+      <c r="B17" t="s" s="7">
         <v>42</v>
-      </c>
-      <c r="B17" t="s" s="7">
-        <v>43</v>
       </c>
       <c r="C17" t="s" s="7">
         <v>8</v>
@@ -1839,10 +1848,10 @@
     </row>
     <row r="18" ht="23.2" customHeight="1">
       <c r="A18" t="s" s="7">
+        <v>43</v>
+      </c>
+      <c r="B18" t="s" s="7">
         <v>44</v>
-      </c>
-      <c r="B18" t="s" s="7">
-        <v>45</v>
       </c>
       <c r="C18" t="s" s="7">
         <v>8</v>
@@ -1860,10 +1869,10 @@
     </row>
     <row r="19" ht="23.2" customHeight="1">
       <c r="A19" t="s" s="7">
+        <v>45</v>
+      </c>
+      <c r="B19" t="s" s="7">
         <v>46</v>
-      </c>
-      <c r="B19" t="s" s="7">
-        <v>47</v>
       </c>
       <c r="C19" t="s" s="7">
         <v>8</v>
@@ -1881,10 +1890,10 @@
     </row>
     <row r="20" ht="23.2" customHeight="1">
       <c r="A20" t="s" s="7">
+        <v>47</v>
+      </c>
+      <c r="B20" t="s" s="7">
         <v>48</v>
-      </c>
-      <c r="B20" t="s" s="7">
-        <v>49</v>
       </c>
       <c r="C20" t="s" s="7">
         <v>8</v>
@@ -1893,19 +1902,19 @@
         <v>9</v>
       </c>
       <c r="E20" t="s" s="7">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="F20" s="8">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="G20" s="9"/>
     </row>
     <row r="21" ht="23.2" customHeight="1">
       <c r="A21" t="s" s="7">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B21" t="s" s="7">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C21" t="s" s="7">
         <v>8</v>
@@ -1914,19 +1923,19 @@
         <v>9</v>
       </c>
       <c r="E21" t="s" s="7">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="F21" s="8">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="G21" s="9"/>
     </row>
     <row r="22" ht="23.2" customHeight="1">
       <c r="A22" t="s" s="7">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B22" t="s" s="7">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C22" t="s" s="7">
         <v>8</v>
@@ -1935,7 +1944,7 @@
         <v>9</v>
       </c>
       <c r="E22" t="s" s="7">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="F22" s="8">
         <v>2023</v>
@@ -1944,10 +1953,10 @@
     </row>
     <row r="23" ht="23.2" customHeight="1">
       <c r="A23" t="s" s="7">
+        <v>54</v>
+      </c>
+      <c r="B23" t="s" s="7">
         <v>55</v>
-      </c>
-      <c r="B23" t="s" s="7">
-        <v>56</v>
       </c>
       <c r="C23" t="s" s="7">
         <v>8</v>
@@ -1956,7 +1965,7 @@
         <v>9</v>
       </c>
       <c r="E23" t="s" s="7">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="F23" s="8">
         <v>2023</v>
@@ -1965,10 +1974,10 @@
     </row>
     <row r="24" ht="23.2" customHeight="1">
       <c r="A24" t="s" s="7">
+        <v>56</v>
+      </c>
+      <c r="B24" t="s" s="7">
         <v>57</v>
-      </c>
-      <c r="B24" t="s" s="7">
-        <v>58</v>
       </c>
       <c r="C24" t="s" s="7">
         <v>8</v>
@@ -1977,7 +1986,7 @@
         <v>9</v>
       </c>
       <c r="E24" t="s" s="7">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="F24" s="8">
         <v>2023</v>
@@ -1986,10 +1995,10 @@
     </row>
     <row r="25" ht="23.2" customHeight="1">
       <c r="A25" t="s" s="7">
+        <v>58</v>
+      </c>
+      <c r="B25" t="s" s="7">
         <v>59</v>
-      </c>
-      <c r="B25" t="s" s="7">
-        <v>60</v>
       </c>
       <c r="C25" t="s" s="7">
         <v>8</v>
@@ -1998,31 +2007,31 @@
         <v>9</v>
       </c>
       <c r="E25" t="s" s="7">
-        <v>10</v>
+        <v>53</v>
       </c>
       <c r="F25" s="8">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="G25" s="9"/>
     </row>
     <row r="26" ht="23.2" customHeight="1">
       <c r="A26" t="s" s="7">
+        <v>60</v>
+      </c>
+      <c r="B26" t="s" s="7">
         <v>61</v>
       </c>
-      <c r="B26" t="s" s="7">
-        <v>60</v>
-      </c>
       <c r="C26" t="s" s="7">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D26" t="s" s="7">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E26" t="s" s="7">
-        <v>10</v>
+        <v>53</v>
       </c>
       <c r="F26" s="8">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="G26" s="9"/>
     </row>
@@ -2118,55 +2127,55 @@
         <v>69</v>
       </c>
       <c r="C31" t="s" s="7">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D31" t="s" s="7">
-        <v>70</v>
+        <v>9</v>
       </c>
       <c r="E31" t="s" s="7">
-        <v>71</v>
+        <v>10</v>
       </c>
       <c r="F31" s="8">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="G31" s="9"/>
     </row>
     <row r="32" ht="23.2" customHeight="1">
       <c r="A32" t="s" s="7">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B32" t="s" s="7">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C32" t="s" s="7">
         <v>12</v>
       </c>
       <c r="D32" t="s" s="7">
-        <v>70</v>
+        <v>13</v>
       </c>
       <c r="E32" t="s" s="7">
-        <v>71</v>
+        <v>10</v>
       </c>
       <c r="F32" s="8">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="G32" s="9"/>
     </row>
     <row r="33" ht="23.2" customHeight="1">
       <c r="A33" t="s" s="7">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B33" t="s" s="7">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C33" t="s" s="7">
         <v>12</v>
       </c>
       <c r="D33" t="s" s="7">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="E33" t="s" s="7">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="F33" s="8">
         <v>2025</v>
@@ -2175,19 +2184,19 @@
     </row>
     <row r="34" ht="23.2" customHeight="1">
       <c r="A34" t="s" s="7">
+        <v>75</v>
+      </c>
+      <c r="B34" t="s" s="7">
         <v>76</v>
-      </c>
-      <c r="B34" t="s" s="7">
-        <v>77</v>
       </c>
       <c r="C34" t="s" s="7">
         <v>12</v>
       </c>
       <c r="D34" t="s" s="7">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="E34" t="s" s="7">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="F34" s="8">
         <v>2025</v>
@@ -2196,19 +2205,19 @@
     </row>
     <row r="35" ht="23.2" customHeight="1">
       <c r="A35" t="s" s="7">
+        <v>77</v>
+      </c>
+      <c r="B35" t="s" s="7">
         <v>78</v>
-      </c>
-      <c r="B35" t="s" s="7">
-        <v>79</v>
       </c>
       <c r="C35" t="s" s="7">
         <v>12</v>
       </c>
       <c r="D35" t="s" s="7">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="E35" t="s" s="7">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="F35" s="8">
         <v>2025</v>
@@ -2217,19 +2226,19 @@
     </row>
     <row r="36" ht="23.2" customHeight="1">
       <c r="A36" t="s" s="7">
+        <v>79</v>
+      </c>
+      <c r="B36" t="s" s="7">
         <v>80</v>
-      </c>
-      <c r="B36" t="s" s="7">
-        <v>81</v>
       </c>
       <c r="C36" t="s" s="7">
         <v>12</v>
       </c>
       <c r="D36" t="s" s="7">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="E36" t="s" s="7">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="F36" s="8">
         <v>2025</v>
@@ -2238,19 +2247,19 @@
     </row>
     <row r="37" ht="23.2" customHeight="1">
       <c r="A37" t="s" s="7">
+        <v>81</v>
+      </c>
+      <c r="B37" t="s" s="7">
         <v>82</v>
       </c>
-      <c r="B37" t="s" s="7">
-        <v>83</v>
-      </c>
       <c r="C37" t="s" s="7">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D37" t="s" s="7">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="E37" t="s" s="7">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="F37" s="8">
         <v>2025</v>
@@ -2259,19 +2268,19 @@
     </row>
     <row r="38" ht="23.2" customHeight="1">
       <c r="A38" t="s" s="7">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B38" t="s" s="7">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C38" t="s" s="7">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D38" t="s" s="7">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="E38" t="s" s="7">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="F38" s="8">
         <v>2025</v>
@@ -2280,19 +2289,19 @@
     </row>
     <row r="39" ht="23.2" customHeight="1">
       <c r="A39" t="s" s="7">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B39" t="s" s="7">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C39" t="s" s="7">
         <v>8</v>
       </c>
       <c r="D39" t="s" s="7">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="E39" t="s" s="7">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F39" s="8">
         <v>2025</v>
@@ -2301,19 +2310,19 @@
     </row>
     <row r="40" ht="23.2" customHeight="1">
       <c r="A40" t="s" s="7">
+        <v>88</v>
+      </c>
+      <c r="B40" t="s" s="7">
         <v>89</v>
-      </c>
-      <c r="B40" t="s" s="7">
-        <v>90</v>
       </c>
       <c r="C40" t="s" s="7">
         <v>8</v>
       </c>
       <c r="D40" t="s" s="7">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="E40" t="s" s="7">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F40" s="8">
         <v>2025</v>
@@ -2322,19 +2331,19 @@
     </row>
     <row r="41" ht="23.2" customHeight="1">
       <c r="A41" t="s" s="7">
+        <v>90</v>
+      </c>
+      <c r="B41" t="s" s="7">
         <v>91</v>
-      </c>
-      <c r="B41" t="s" s="7">
-        <v>92</v>
       </c>
       <c r="C41" t="s" s="7">
         <v>8</v>
       </c>
       <c r="D41" t="s" s="7">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="E41" t="s" s="7">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F41" s="8">
         <v>2025</v>
@@ -2342,21 +2351,45 @@
       <c r="G41" s="9"/>
     </row>
     <row r="42" ht="23.2" customHeight="1">
-      <c r="A42" s="9"/>
-      <c r="B42" s="9"/>
-      <c r="C42" s="9"/>
-      <c r="D42" s="9"/>
-      <c r="E42" s="9"/>
-      <c r="F42" s="9"/>
+      <c r="A42" t="s" s="7">
+        <v>92</v>
+      </c>
+      <c r="B42" t="s" s="7">
+        <v>93</v>
+      </c>
+      <c r="C42" t="s" s="7">
+        <v>8</v>
+      </c>
+      <c r="D42" t="s" s="7">
+        <v>73</v>
+      </c>
+      <c r="E42" t="s" s="7">
+        <v>87</v>
+      </c>
+      <c r="F42" s="8">
+        <v>2025</v>
+      </c>
       <c r="G42" s="9"/>
     </row>
     <row r="43" ht="23.2" customHeight="1">
-      <c r="A43" s="9"/>
-      <c r="B43" s="9"/>
-      <c r="C43" s="9"/>
-      <c r="D43" s="9"/>
-      <c r="E43" s="9"/>
-      <c r="F43" s="9"/>
+      <c r="A43" t="s" s="7">
+        <v>94</v>
+      </c>
+      <c r="B43" t="s" s="7">
+        <v>95</v>
+      </c>
+      <c r="C43" t="s" s="7">
+        <v>8</v>
+      </c>
+      <c r="D43" t="s" s="7">
+        <v>73</v>
+      </c>
+      <c r="E43" t="s" s="7">
+        <v>87</v>
+      </c>
+      <c r="F43" s="8">
+        <v>2025</v>
+      </c>
       <c r="G43" s="9"/>
     </row>
     <row r="44" ht="23.2" customHeight="1">
@@ -2368,6 +2401,24 @@
       <c r="F44" s="9"/>
       <c r="G44" s="9"/>
     </row>
+    <row r="45" ht="23.2" customHeight="1">
+      <c r="A45" s="9"/>
+      <c r="B45" s="9"/>
+      <c r="C45" s="9"/>
+      <c r="D45" s="9"/>
+      <c r="E45" s="9"/>
+      <c r="F45" s="9"/>
+      <c r="G45" s="9"/>
+    </row>
+    <row r="46" ht="23.2" customHeight="1">
+      <c r="A46" s="9"/>
+      <c r="B46" s="9"/>
+      <c r="C46" s="9"/>
+      <c r="D46" s="9"/>
+      <c r="E46" s="9"/>
+      <c r="F46" s="9"/>
+      <c r="G46" s="9"/>
+    </row>
   </sheetData>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.277778" footer="0.277778"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="72" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>

</xml_diff>